<commit_message>
xlsx changed to sheets. button that goes to next match.
</commit_message>
<xml_diff>
--- a/prode_data.xlsx
+++ b/prode_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Desktop\prode26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB755397-C5C3-404C-AD61-4596CC8E2746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B777908A-5F16-4DC2-A9A0-6A40482E0541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="780" firstSheet="1" activeTab="8" xr2:uid="{E90A7C8B-E6B4-4E6A-9703-A59097F09DC3}"/>
   </bookViews>
@@ -1075,11 +1075,11 @@
       </c>
       <c r="F4" s="1">
         <f>+SUM('group-stage-3'!J2:J25,'group-stage-3'!M2:M25)</f>
-        <v>16.3</v>
+        <v>20.3</v>
       </c>
       <c r="G4" s="1">
         <f>+SUM('group-stage-3'!K2:K25,'group-stage-3'!O2:O25)</f>
-        <v>18.3</v>
+        <v>19.3</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1177,11 +1177,11 @@
       </c>
       <c r="F10" s="1">
         <f>+SUM(F2:F9)</f>
-        <v>61.400000000000006</v>
+        <v>65.400000000000006</v>
       </c>
       <c r="G10" s="1">
         <f>+SUM(G2:G9)</f>
-        <v>57.3</v>
+        <v>58.3</v>
       </c>
     </row>
   </sheetData>
@@ -7498,15 +7498,19 @@
       <c r="G18" s="15">
         <v>1</v>
       </c>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="K18" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="H18" s="19">
+        <v>1</v>
+      </c>
+      <c r="I18" s="19">
+        <v>1</v>
+      </c>
+      <c r="J18" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K18" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="L18" s="11"/>
       <c r="M18" s="11"/>
@@ -7535,15 +7539,19 @@
       <c r="G19" s="15">
         <v>2</v>
       </c>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="K19" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="H19" s="19">
+        <v>1</v>
+      </c>
+      <c r="I19" s="19">
+        <v>5</v>
+      </c>
+      <c r="J19" s="11">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K19" s="15">
+        <f t="shared" si="1"/>
+        <v>1</v>
       </c>
       <c r="L19" s="11"/>
       <c r="M19" s="11"/>

</xml_diff>